<commit_message>
se terminaron los arreglos para casi la version final sin las herramientas del hardware
</commit_message>
<xml_diff>
--- a/reportes/inventario.xlsx
+++ b/reportes/inventario.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,7 +430,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>uniforme de gala</v>
+        <v>gala</v>
       </c>
       <c r="B2" t="str">
         <v>Uniformes</v>
@@ -445,21 +445,21 @@
         <v>L</v>
       </c>
       <c r="F2">
-        <v>50000</v>
+        <v>130000</v>
       </c>
       <c r="G2">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H2">
         <v>3</v>
       </c>
       <c r="I2" t="str">
-        <v>1000010001NaN</v>
+        <v>1000010002NaN</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>uniforme de gala</v>
+        <v>gala</v>
       </c>
       <c r="B3" t="str">
         <v>Uniformes</v>
@@ -474,21 +474,50 @@
         <v>M</v>
       </c>
       <c r="F3">
-        <v>48000</v>
+        <v>120000</v>
       </c>
       <c r="G3">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H3">
         <v>3</v>
       </c>
       <c r="I3" t="str">
-        <v>1000010002NaN</v>
+        <v>1000010001NaN</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>gala</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Uniformes</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Guanenta</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Hombre</v>
+      </c>
+      <c r="E4" t="str">
+        <v>S</v>
+      </c>
+      <c r="F4">
+        <v>110000</v>
+      </c>
+      <c r="G4">
+        <v>48</v>
+      </c>
+      <c r="H4">
+        <v>3</v>
+      </c>
+      <c r="I4" t="str">
+        <v>1000010003NaN</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: :sparkles: arregleé bugs, cambié estetica y puse mas opciones requeridas
agregué la opcion de pago en efectivo o transferencia, cambié la estetica completamente dando mas profesionalismon mejoré metas y reportes para poder tener toda la informacion
</commit_message>
<xml_diff>
--- a/reportes/inventario.xlsx
+++ b/reportes/inventario.xlsx
@@ -6022,7 +6022,7 @@
         <v>0</v>
       </c>
       <c r="H176">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I176">
         <v>8</v>
@@ -6502,7 +6502,7 @@
         <v>0</v>
       </c>
       <c r="H191">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I191">
         <v>8</v>
@@ -8102,7 +8102,7 @@
         <v>0</v>
       </c>
       <c r="H241">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I241">
         <v>8</v>

</xml_diff>